<commit_message>
Repair seed Excel files as valid XLSX
</commit_message>
<xml_diff>
--- a/library/seed/01_Wuthering_Waves.xlsx
+++ b/library/seed/01_Wuthering_Waves.xlsx
@@ -1,1621 +1,1226 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Characters" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Имя персонажа</t>
+          <t xml:space="preserve">Имя персонажа</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Стихия</t>
+          <t xml:space="preserve">Стихия</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Редкость</t>
+          <t xml:space="preserve">Редкость</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t xml:space="preserve">1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sigrika</t>
+          <t xml:space="preserve">Sigrika</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t xml:space="preserve">1.2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Luuk Herssen</t>
+          <t xml:space="preserve">Luuk Herssen</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t xml:space="preserve">1.3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mornye</t>
+          <t xml:space="preserve">Mornye</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t xml:space="preserve">1.4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Roccia</t>
+          <t xml:space="preserve">Roccia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t xml:space="preserve">1.5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lynae</t>
+          <t xml:space="preserve">Lynae</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t xml:space="preserve">1.6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aalto</t>
+          <t xml:space="preserve">Aalto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t xml:space="preserve">1.7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Augusta</t>
+          <t xml:space="preserve">Augusta</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t xml:space="preserve">1.8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Baizhi</t>
+          <t xml:space="preserve">Baizhi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t xml:space="preserve">1.9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Buling</t>
+          <t xml:space="preserve">Buling</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t xml:space="preserve">1.10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Brant</t>
+          <t xml:space="preserve">Brant</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t xml:space="preserve">1.11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Camellya</t>
+          <t xml:space="preserve">Camellya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t xml:space="preserve">1.12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cantarella</t>
+          <t xml:space="preserve">Cantarella</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t xml:space="preserve">1.13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Carlotta</t>
+          <t xml:space="preserve">Carlotta</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t xml:space="preserve">1.14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Changli</t>
+          <t xml:space="preserve">Changli</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t xml:space="preserve">1.15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shorekeeper</t>
+          <t xml:space="preserve">Shorekeeper</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t xml:space="preserve">1.16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lumi</t>
+          <t xml:space="preserve">Lumi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t xml:space="preserve">1.17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Phoebe</t>
+          <t xml:space="preserve">Phoebe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t xml:space="preserve">1.18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Xiangli Yao</t>
+          <t xml:space="preserve">Xiangli Yao</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t xml:space="preserve">1.19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Youhu</t>
+          <t xml:space="preserve">Youhu</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t xml:space="preserve">1.20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Zani</t>
+          <t xml:space="preserve">Zani</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t xml:space="preserve">1.21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Zhezhi</t>
+          <t xml:space="preserve">Zhezhi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t xml:space="preserve">1.22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cartethyia</t>
+          <t xml:space="preserve">Cartethyia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t xml:space="preserve">1.23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Chisa</t>
+          <t xml:space="preserve">Chisa</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t xml:space="preserve">1.24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chixia</t>
+          <t xml:space="preserve">Chixia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t xml:space="preserve">1.25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ciaccona</t>
+          <t xml:space="preserve">Ciaccona</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t xml:space="preserve">1.26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Danjin</t>
+          <t xml:space="preserve">Danjin</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t xml:space="preserve">1.27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Denia</t>
+          <t xml:space="preserve">Denia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t xml:space="preserve">1.28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Encore</t>
+          <t xml:space="preserve">Encore</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t xml:space="preserve">1.29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Galbrena</t>
+          <t xml:space="preserve">Galbrena</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t xml:space="preserve">1.30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hiyuki</t>
+          <t xml:space="preserve">Hiyuki</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t xml:space="preserve">1.31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hsin</t>
+          <t xml:space="preserve">Hsin</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t xml:space="preserve">1.32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Iuno</t>
+          <t xml:space="preserve">Iuno</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t xml:space="preserve">1.33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jianxin</t>
+          <t xml:space="preserve">Jianxin</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t xml:space="preserve">1.34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jinhsi</t>
+          <t xml:space="preserve">Jinhsi</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t xml:space="preserve">1.35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jingran</t>
+          <t xml:space="preserve">Jingran</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t xml:space="preserve">1.36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jiyan</t>
+          <t xml:space="preserve">Jiyan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t xml:space="preserve">1.37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Lingyang</t>
+          <t xml:space="preserve">Lingyang</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t xml:space="preserve">1.38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Lupa</t>
+          <t xml:space="preserve">Lupa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t xml:space="preserve">1.39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lucy</t>
+          <t xml:space="preserve">Lucy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t xml:space="preserve">1.40</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Aemeath</t>
+          <t xml:space="preserve">Aemeath</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t xml:space="preserve">1.41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mortefi</t>
+          <t xml:space="preserve">Mortefi</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t xml:space="preserve">1.42</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Phrolova</t>
+          <t xml:space="preserve">Phrolova</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t xml:space="preserve">1.43</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Qiuyuan</t>
+          <t xml:space="preserve">Qiuyuan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t xml:space="preserve">1.44</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Qingxiao</t>
+          <t xml:space="preserve">Qingxiao</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t xml:space="preserve">1.45</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Rebecca</t>
+          <t xml:space="preserve">Rebecca</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t xml:space="preserve">1.46</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sanhua</t>
+          <t xml:space="preserve">Sanhua</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t xml:space="preserve">1.47</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Suisui</t>
+          <t xml:space="preserve">Suisui</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t xml:space="preserve">1.48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Suoming</t>
+          <t xml:space="preserve">Suoming</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t xml:space="preserve">1.49</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Taoqi</t>
+          <t xml:space="preserve">Taoqi</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t xml:space="preserve">1.50</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Verina</t>
+          <t xml:space="preserve">Verina</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t xml:space="preserve">1.51</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yangyang</t>
+          <t xml:space="preserve">Yangyang</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t xml:space="preserve">1.52</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yangyang: Xuanling</t>
+          <t xml:space="preserve">Yangyang: Xuanling</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t xml:space="preserve">1.53</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yinlin</t>
+          <t xml:space="preserve">Yinlin</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t xml:space="preserve">1.54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yuanwu</t>
+          <t xml:space="preserve">Yuanwu</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync character library and ID portraits
</commit_message>
<xml_diff>
--- a/library/seed/01_Wuthering_Waves.xlsx
+++ b/library/seed/01_Wuthering_Waves.xlsx
@@ -1,1226 +1,1619 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Characters" sheetId="1" r:id="rId1"/>
+    <sheet name="Characters" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">ID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Имя персонажа</t>
+          <t>Имя персонажа</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Стихия</t>
+          <t>Стихия</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Редкость</t>
+          <t>Редкость</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sigrika</t>
+          <t>Sigrika</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.2</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luuk Herssen</t>
+          <t>Luuk Herssen</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.3</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mornye</t>
+          <t>Mornye</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.4</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Roccia</t>
+          <t>Roccia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.5</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lynae</t>
+          <t>Lynae</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.6</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aalto</t>
+          <t>Aalto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.7</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Augusta</t>
+          <t>Augusta</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.8</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baizhi</t>
+          <t>Baizhi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.9</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buling</t>
+          <t>Buling</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.10</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brant</t>
+          <t>Brant</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.11</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Camellya</t>
+          <t>Camellya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.12</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cantarella</t>
+          <t>Cantarella</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.13</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carlotta</t>
+          <t>Carlotta</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.14</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Changli</t>
+          <t>Changli</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.15</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shorekeeper</t>
+          <t>Shorekeeper</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.16</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lumi</t>
+          <t>Lumi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.17</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoebe</t>
+          <t>Phoebe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.18</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xiangli Yao</t>
+          <t>Xiangli Yao</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.19</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Youhu</t>
+          <t>Youhu</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.20</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zani</t>
+          <t>Zani</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.21</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zhezhi</t>
+          <t>Zhezhi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.22</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cartethyia</t>
+          <t>Cartethyia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.23</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chisa</t>
+          <t>Chisa</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.24</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chixia</t>
+          <t>Chixia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.25</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ciaccona</t>
+          <t>Ciaccona</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.26</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Danjin</t>
+          <t>Danjin</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.27</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Denia</t>
+          <t>Denia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.28</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Encore</t>
+          <t>Encore</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.29</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Galbrena</t>
+          <t>Galbrena</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.30</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hiyuki</t>
+          <t>Hiyuki</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.31</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hsin</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
+          <t>Hsin</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.32</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iuno</t>
+          <t>Iuno</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.33</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jianxin</t>
+          <t>Jianxin</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.34</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jinhsi</t>
+          <t>Jinhsi</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.35</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jingran</t>
+          <t>Jingran</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.36</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jiyan</t>
+          <t>Jiyan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.37</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lingyang</t>
+          <t>Lingyang</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.38</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lupa</t>
+          <t>Lupa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.39</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lucy</t>
+          <t>Lucy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.40</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aemeath</t>
+          <t>Aemeath</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.41</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mortefi</t>
+          <t>Mortefi</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fusion</t>
+          <t>Fusion</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.42</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phrolova</t>
+          <t>Phrolova</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.43</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qiuyuan</t>
+          <t>Qiuyuan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.44</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qingxiao</t>
+          <t>Qingxiao</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.45</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rebecca</t>
+          <t>Rebecca</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.46</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sanhua</t>
+          <t>Sanhua</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.47</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suisui</t>
+          <t>Suisui</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glacio</t>
+          <t>Glacio</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.48</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suoming</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
+          <t>Suoming</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.49</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Taoqi</t>
+          <t>Taoqi</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.50</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verina</t>
+          <t>Verina</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spectro</t>
+          <t>Spectro</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.51</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yangyang</t>
+          <t>Yangyang</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aero</t>
+          <t>Aero</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.52</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yangyang: Xuanling</t>
+          <t>Yangyang: Xuanling</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Havoc</t>
+          <t>Havoc</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.53</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yinlin</t>
+          <t>Yinlin</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">5★</t>
+          <t>5★</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.54</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yuanwu</t>
+          <t>Yuanwu</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electro</t>
+          <t>Electro</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">4★</t>
+          <t>4★</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Admin: update Wuthering Waves character database
</commit_message>
<xml_diff>
--- a/library/seed/01_Wuthering_Waves.xlsx
+++ b/library/seed/01_Wuthering_Waves.xlsx
@@ -1,1619 +1,1243 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Characters" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t xml:space="preserve">ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Имя персонажа</t>
+          <t xml:space="preserve">Имя персонажа</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Стихия</t>
+          <t xml:space="preserve">Стихия</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Редкость</t>
+          <t xml:space="preserve">Редкость</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t xml:space="preserve">1.1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sigrika</t>
+          <t xml:space="preserve">Sigrika</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t xml:space="preserve">1.2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Luuk Herssen</t>
+          <t xml:space="preserve">Luuk Herssen</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t xml:space="preserve">1.3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Mornye</t>
+          <t xml:space="preserve">Mornye</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t xml:space="preserve">1.4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Roccia</t>
+          <t xml:space="preserve">Roccia</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t xml:space="preserve">1.5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lynae</t>
+          <t xml:space="preserve">Lynae</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t xml:space="preserve">1.6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aalto</t>
+          <t xml:space="preserve">Aalto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t xml:space="preserve">1.7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Augusta</t>
+          <t xml:space="preserve">Augusta</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t xml:space="preserve">1.8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Baizhi</t>
+          <t xml:space="preserve">Baizhi</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t xml:space="preserve">1.9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Buling</t>
+          <t xml:space="preserve">Buling</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t xml:space="preserve">1.10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Brant</t>
+          <t xml:space="preserve">Brant</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t xml:space="preserve">1.11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Camellya</t>
+          <t xml:space="preserve">Camellya</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t xml:space="preserve">1.12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cantarella</t>
+          <t xml:space="preserve">Cantarella</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t xml:space="preserve">1.13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Carlotta</t>
+          <t xml:space="preserve">Carlotta</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t xml:space="preserve">1.14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Changli</t>
+          <t xml:space="preserve">Changli</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t xml:space="preserve">1.15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Shorekeeper</t>
+          <t xml:space="preserve">Shorekeeper</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t xml:space="preserve">1.16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Lumi</t>
+          <t xml:space="preserve">Lumi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t xml:space="preserve">1.17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Phoebe</t>
+          <t xml:space="preserve">Phoebe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t xml:space="preserve">1.18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Xiangli Yao</t>
+          <t xml:space="preserve">Xiangli Yao</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t xml:space="preserve">1.19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Youhu</t>
+          <t xml:space="preserve">Youhu</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t xml:space="preserve">1.20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Zani</t>
+          <t xml:space="preserve">Zani</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t xml:space="preserve">1.21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Zhezhi</t>
+          <t xml:space="preserve">Zhezhi</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t xml:space="preserve">1.22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cartethyia</t>
+          <t xml:space="preserve">Cartethyia</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t xml:space="preserve">1.23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Chisa</t>
+          <t xml:space="preserve">Chisa</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t xml:space="preserve">1.24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chixia</t>
+          <t xml:space="preserve">Chixia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t xml:space="preserve">1.25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ciaccona</t>
+          <t xml:space="preserve">Ciaccona</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t xml:space="preserve">1.26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Danjin</t>
+          <t xml:space="preserve">Danjin</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t xml:space="preserve">1.27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Denia</t>
+          <t xml:space="preserve">Denia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t xml:space="preserve">1.28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Encore</t>
+          <t xml:space="preserve">Encore</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t xml:space="preserve">1.29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Galbrena</t>
+          <t xml:space="preserve">Galbrena</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t xml:space="preserve">1.30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Hiyuki</t>
+          <t xml:space="preserve">Hiyuki</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t xml:space="preserve">1.31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hsin</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
+          <t xml:space="preserve">Hsin</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t xml:space="preserve">1.32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Iuno</t>
+          <t xml:space="preserve">Iuno</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t xml:space="preserve">1.33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jianxin</t>
+          <t xml:space="preserve">Jianxin</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t xml:space="preserve">1.34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jinhsi</t>
+          <t xml:space="preserve">Jinhsi</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t xml:space="preserve">1.35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jingran</t>
+          <t xml:space="preserve">Jingran</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t xml:space="preserve">1.36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jiyan</t>
+          <t xml:space="preserve">Jiyan</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t xml:space="preserve">1.37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Lingyang</t>
+          <t xml:space="preserve">Lingyang</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t xml:space="preserve">1.38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Lupa</t>
+          <t xml:space="preserve">Lupa</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t xml:space="preserve">1.39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Lucy</t>
+          <t xml:space="preserve">Lucy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t xml:space="preserve">1.40</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Aemeath</t>
+          <t xml:space="preserve">Aemeath</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t xml:space="preserve">1.41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Mortefi</t>
+          <t xml:space="preserve">Mortefi</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Fusion</t>
+          <t xml:space="preserve">Fusion</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t xml:space="preserve">1.42</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Phrolova</t>
+          <t xml:space="preserve">Phrolova</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t xml:space="preserve">1.43</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Qiuyuan</t>
+          <t xml:space="preserve">Qiuyuan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t xml:space="preserve">1.44</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Qingxiao</t>
+          <t xml:space="preserve">Qingxiao</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t xml:space="preserve">1.45</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Rebecca</t>
+          <t xml:space="preserve">Rebecca</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t xml:space="preserve">1.46</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sanhua</t>
+          <t xml:space="preserve">Sanhua</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t xml:space="preserve">1.47</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Suisui</t>
+          <t xml:space="preserve">Suisui</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Glacio</t>
+          <t xml:space="preserve">Glacio</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t xml:space="preserve">1.48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Suoming</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
+          <t xml:space="preserve">Suoming</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t xml:space="preserve">1.49</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Taoqi</t>
+          <t xml:space="preserve">Taoqi</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t xml:space="preserve">1.50</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Verina</t>
+          <t xml:space="preserve">Verina</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Spectro</t>
+          <t xml:space="preserve">Spectro</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t xml:space="preserve">1.51</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Yangyang</t>
+          <t xml:space="preserve">Yangyang</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Aero</t>
+          <t xml:space="preserve">Aero</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t xml:space="preserve">1.52</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Yangyang: Xuanling</t>
+          <t xml:space="preserve">Yangyang: Xuanling</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Havoc</t>
+          <t xml:space="preserve">Havoc</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t xml:space="preserve">1.53</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Yinlin</t>
+          <t xml:space="preserve">Yinlin</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>5★</t>
+          <t xml:space="preserve">5★</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t xml:space="preserve">1.54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Yuanwu</t>
+          <t xml:space="preserve">Yuanwu</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Electro</t>
+          <t xml:space="preserve">Electro</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>4★</t>
+          <t xml:space="preserve">4★</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>